<commit_message>
protocolo de seguridad y robustez, se va  a implementar.
</commit_message>
<xml_diff>
--- a/2026_09_contratacion_automata.xlsx
+++ b/2026_09_contratacion_automata.xlsx
@@ -414,600 +414,608 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DI2"/>
+  <dimension ref="A1:DK2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>numero de identidad del contratado</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sujeto</t>
+          <t>nombre del contratado</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>entidad</t>
+          <t>ruta_carpeta</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>cliente</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>asesor</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>documento_id_existe</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>documento_id_numeroid</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>documento_id_nombre</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>documento_id_tipo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>contrato_laboral_existe</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>contrato_laboral_numeroid</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>contrato_laboral_nombre</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>contrato_laboral_fecha</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>contrato_laboral_firma</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>curso_etica_existe</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>curso_etica_numeroid</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>curso_etica_nombre</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>curso_etica_titulo</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>curso_cultura_existe</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>curso_cultura_numeroid</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>curso_cultura_nombre</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>curso_cultura_titulo</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>curso_transparencia_existe</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>curso_transparencia_numeroid</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>curso_transparencia_nombre</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>curso_transparencia_titulo</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>curso_otro_existe</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>curso_otro_numeroid</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>curso_otro_nombre</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>curso_otro_titulo</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>pruebas_psicotecnicas_existe</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>pruebas_psicotecnicas_numeroid</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>pruebas_psicotecnicas_nombre</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>verificacion_referencias_existe</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>verificacion_referencias_numeroid</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>verificacion_referencias_nombre</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>arl_existe</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>arl_numeroid</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>arl_nombre</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ccf_existe</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>ccf_numeroid</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>ccf_nombre</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>examen_medico_ingreso_existe</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>examen_medico_ingreso_numeroid</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>examen_medico_ingreso_nombre</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>antecedente_policia_existe</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>antecedente_policia_numeroid</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>antecedente_policia_nombre</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>antecedente_policia_resultado</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>antecedente_procuraduria_existe</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>antecedente_procuraduria_numeroid</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>antecedente_procuraduria_nombre</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>antecedente_procuraduria_resultado</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>antecedente_contraloria_existe</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>antecedente_contraloria_numeroid</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>antecedente_contraloria_nombre</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>antecedente_contraloria_resultado</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>cuenta_bancaria_existe</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>cuenta_bancaria_numeroid</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>cuenta_bancaria_nombre</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>cuenta_bancaria_numero</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>pension_o_cesantias_existe</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>pension_o_cesantias_numeroid</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>pension_o_cesantias_nombre</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>pension_o_cesantias_tipo</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>eps_o_adres_existe</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>eps_o_adres_numeroid</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>eps_o_adres_nombre</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>estudios_existe</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>estudios_numeroid</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>estudios_nombre</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>estudios_bachillerato</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>referencia_personal_existe</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>referencia_personal_numeroid</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>referencia_personal_nombre</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>referencia_laboral_existe</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>referencia_laboral_numeroid</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>referencia_laboral_nombre</t>
         </is>
       </c>
-      <c r="BY1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>hoja_de_vida_existe</t>
         </is>
       </c>
-      <c r="BZ1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>hoja_de_vida_numeroid</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>hoja_de_vida_nombre</t>
         </is>
       </c>
-      <c r="CB1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_existe</t>
         </is>
       </c>
-      <c r="CC1" t="inlineStr">
+      <c r="CE1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_numeroid</t>
         </is>
       </c>
-      <c r="CD1" t="inlineStr">
+      <c r="CF1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_nombre</t>
         </is>
       </c>
-      <c r="CE1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_hojas</t>
         </is>
       </c>
-      <c r="CF1" t="inlineStr">
+      <c r="CH1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_firmas</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CI1" t="inlineStr">
         <is>
           <t>informe_datacredito_existe</t>
         </is>
       </c>
-      <c r="CH1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
         <is>
           <t>informe_datacredito_numeroid</t>
         </is>
       </c>
-      <c r="CI1" t="inlineStr">
+      <c r="CK1" t="inlineStr">
         <is>
           <t>informe_datacredito_nombre</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CL1" t="inlineStr">
         <is>
           <t>informe_datacredito_moras</t>
         </is>
       </c>
-      <c r="CK1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>informe_datacredito_demandas</t>
         </is>
       </c>
-      <c r="CL1" t="inlineStr">
+      <c r="CN1" t="inlineStr">
         <is>
           <t>informe_bases_existe</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
+      <c r="CO1" t="inlineStr">
         <is>
           <t>informe_bases_numeroid</t>
         </is>
       </c>
-      <c r="CN1" t="inlineStr">
+      <c r="CP1" t="inlineStr">
         <is>
           <t>informe_bases_nombre</t>
         </is>
       </c>
-      <c r="CO1" t="inlineStr">
+      <c r="CQ1" t="inlineStr">
         <is>
           <t>informe_bases_inconveniente</t>
         </is>
       </c>
-      <c r="CP1" t="inlineStr">
+      <c r="CR1" t="inlineStr">
         <is>
           <t>visita_domiciliaria_existe</t>
         </is>
       </c>
-      <c r="CQ1" t="inlineStr">
+      <c r="CS1" t="inlineStr">
         <is>
           <t>visita_domiciliaria_numeroid</t>
         </is>
       </c>
-      <c r="CR1" t="inlineStr">
+      <c r="CT1" t="inlineStr">
         <is>
           <t>visita_domiciliaria_nombre</t>
         </is>
       </c>
-      <c r="CS1" t="inlineStr">
+      <c r="CU1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_existe</t>
         </is>
       </c>
-      <c r="CT1" t="inlineStr">
+      <c r="CV1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_numeroid</t>
         </is>
       </c>
-      <c r="CU1" t="inlineStr">
+      <c r="CW1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_nombre</t>
         </is>
       </c>
-      <c r="CV1" t="inlineStr">
+      <c r="CX1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_firma</t>
         </is>
       </c>
-      <c r="CW1" t="inlineStr">
+      <c r="CY1" t="inlineStr">
         <is>
           <t>checklist_documentos_existe</t>
         </is>
       </c>
-      <c r="CX1" t="inlineStr">
+      <c r="CZ1" t="inlineStr">
         <is>
           <t>checklist_documentos_numeroid</t>
         </is>
       </c>
-      <c r="CY1" t="inlineStr">
+      <c r="DA1" t="inlineStr">
         <is>
           <t>checklist_documentos_nombre</t>
         </is>
       </c>
-      <c r="CZ1" t="inlineStr">
+      <c r="DB1" t="inlineStr">
         <is>
           <t>manual_de_funciones_existe</t>
         </is>
       </c>
-      <c r="DA1" t="inlineStr">
+      <c r="DC1" t="inlineStr">
         <is>
           <t>manual_de_funciones_numeroid</t>
         </is>
       </c>
-      <c r="DB1" t="inlineStr">
+      <c r="DD1" t="inlineStr">
         <is>
           <t>manual_de_funciones_nombre</t>
         </is>
       </c>
-      <c r="DC1" t="inlineStr">
+      <c r="DE1" t="inlineStr">
         <is>
           <t>compilado_existe</t>
         </is>
       </c>
-      <c r="DD1" t="inlineStr">
+      <c r="DF1" t="inlineStr">
         <is>
           <t>compilado_numeroid</t>
         </is>
       </c>
-      <c r="DE1" t="inlineStr">
+      <c r="DG1" t="inlineStr">
         <is>
           <t>compilado_nombre</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="DH1" t="inlineStr">
         <is>
           <t>otros_existe</t>
         </is>
       </c>
-      <c r="DG1" t="inlineStr">
+      <c r="DI1" t="inlineStr">
         <is>
           <t>otros_numeroid</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="DJ1" t="inlineStr">
         <is>
           <t>otros_nombre</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="DK1" t="inlineStr">
         <is>
           <t>otros_comentario</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1121877026</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1121877026</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1121877026 GARCIA LOPEZ NATHALY</t>
+          <t>GARCIA LOPEZ NATHALY</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>/home/real_home/videodrome_estudio/desarrollo/tmp_automatizacion/TEMP/BANCO_DE_BOGOTA_JUNIO_2026/ALEXANDRA BARRERA/1121877026 GARCIA LOPEZ NATHALY</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>ALEXANDRA BARRERA</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>BANCO_DE_BOGOTA_JUNIO_2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1017,19 +1025,19 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>CC</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1037,19 +1045,19 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>20260616</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1062,19 +1070,19 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
           <t>CÓDIGO DE ÉTICA Y CONDUCTA - SAGRILAFT</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1082,19 +1090,19 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>INDUCCIÓN CULTURA SALESLAND</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="W2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1102,41 +1110,41 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
           <t>PROGRAMA DE TRANSPARENCIA Y ÉTICA EMPRESARIAL</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr">
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr">
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1189,19 +1197,19 @@
       </c>
       <c r="AU2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="AX2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1209,39 +1217,39 @@
       </c>
       <c r="AY2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="BB2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr">
+      <c r="BE2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="BF2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1249,19 +1257,19 @@
       </c>
       <c r="BG2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
           <t>445595770</t>
         </is>
       </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="BJ2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1269,19 +1277,19 @@
       </c>
       <c r="BK2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
           <t>PENSIONES Y CESANTIAS</t>
         </is>
       </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BM2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="BN2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1304,121 +1312,121 @@
       </c>
       <c r="BR2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
           <t>BACHILLERATO</t>
         </is>
       </c>
-      <c r="BS2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BT2" t="inlineStr">
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>SIN_DATOS</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CF2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CG2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CH2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CI2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="BU2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BY2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CE2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CF2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CG2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="CH2" t="inlineStr"/>
-      <c r="CI2" t="inlineStr"/>
       <c r="CJ2" t="inlineStr"/>
       <c r="CK2" t="inlineStr"/>
-      <c r="CL2" t="inlineStr">
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
       <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr">
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr">
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
       <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="CX2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="CW2" t="inlineStr"/>
+      <c r="CX2" t="inlineStr"/>
       <c r="CY2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1441,19 +1449,29 @@
       </c>
       <c r="DC2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DD2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DE2" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="DD2" t="inlineStr"/>
-      <c r="DE2" t="inlineStr"/>
-      <c r="DF2" t="inlineStr">
+      <c r="DF2" t="inlineStr"/>
+      <c r="DG2" t="inlineStr"/>
+      <c r="DH2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="DG2" t="inlineStr"/>
-      <c r="DH2" t="inlineStr"/>
       <c r="DI2" t="inlineStr"/>
+      <c r="DJ2" t="inlineStr"/>
+      <c r="DK2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
automata completo, version 0.0.1
</commit_message>
<xml_diff>
--- a/2026_09_contratacion_automata.xlsx
+++ b/2026_09_contratacion_automata.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DK2"/>
+  <dimension ref="A1:DP2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -725,270 +725,295 @@
       </c>
       <c r="BJ1" t="inlineStr">
         <is>
-          <t>pension_o_cesantias_existe</t>
+          <t>pension_y_cesantias_existe</t>
         </is>
       </c>
       <c r="BK1" t="inlineStr">
         <is>
-          <t>pension_o_cesantias_numeroid</t>
+          <t>pension_y_cesantias_numeroid</t>
         </is>
       </c>
       <c r="BL1" t="inlineStr">
         <is>
-          <t>pension_o_cesantias_nombre</t>
+          <t>pension_y_cesantias_nombre</t>
         </is>
       </c>
       <c r="BM1" t="inlineStr">
         <is>
-          <t>pension_o_cesantias_tipo</t>
+          <t>prensiones_existe</t>
         </is>
       </c>
       <c r="BN1" t="inlineStr">
         <is>
+          <t>prensiones_numeroid</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>prensiones_nombre</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>cesantias_existe</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>cesantias_numeroid</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>cesantias_nombre</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
           <t>eps_o_adres_existe</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>eps_o_adres_numeroid</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>eps_o_adres_nombre</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>estudios_existe</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>estudios_numeroid</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>estudios_nombre</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>estudios_bachillerato</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>referencia_personal_existe</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>referencia_personal_numeroid</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>referencia_personal_nombre</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>referencia_laboral_existe</t>
         </is>
       </c>
-      <c r="BY1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>referencia_laboral_numeroid</t>
         </is>
       </c>
-      <c r="BZ1" t="inlineStr">
+      <c r="CE1" t="inlineStr">
         <is>
           <t>referencia_laboral_nombre</t>
         </is>
       </c>
-      <c r="CA1" t="inlineStr">
+      <c r="CF1" t="inlineStr">
         <is>
           <t>hoja_de_vida_existe</t>
         </is>
       </c>
-      <c r="CB1" t="inlineStr">
+      <c r="CG1" t="inlineStr">
         <is>
           <t>hoja_de_vida_numeroid</t>
         </is>
       </c>
-      <c r="CC1" t="inlineStr">
+      <c r="CH1" t="inlineStr">
         <is>
           <t>hoja_de_vida_nombre</t>
         </is>
       </c>
-      <c r="CD1" t="inlineStr">
+      <c r="CI1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_existe</t>
         </is>
       </c>
-      <c r="CE1" t="inlineStr">
+      <c r="CJ1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_numeroid</t>
         </is>
       </c>
-      <c r="CF1" t="inlineStr">
+      <c r="CK1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_nombre</t>
         </is>
       </c>
-      <c r="CG1" t="inlineStr">
+      <c r="CL1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_hojas</t>
         </is>
       </c>
-      <c r="CH1" t="inlineStr">
+      <c r="CM1" t="inlineStr">
         <is>
           <t>formatos_para_la_contratacion_firmas</t>
         </is>
       </c>
-      <c r="CI1" t="inlineStr">
+      <c r="CN1" t="inlineStr">
         <is>
           <t>informe_datacredito_existe</t>
         </is>
       </c>
-      <c r="CJ1" t="inlineStr">
+      <c r="CO1" t="inlineStr">
         <is>
           <t>informe_datacredito_numeroid</t>
         </is>
       </c>
-      <c r="CK1" t="inlineStr">
+      <c r="CP1" t="inlineStr">
         <is>
           <t>informe_datacredito_nombre</t>
         </is>
       </c>
-      <c r="CL1" t="inlineStr">
+      <c r="CQ1" t="inlineStr">
         <is>
           <t>informe_datacredito_moras</t>
         </is>
       </c>
-      <c r="CM1" t="inlineStr">
+      <c r="CR1" t="inlineStr">
         <is>
           <t>informe_datacredito_demandas</t>
         </is>
       </c>
-      <c r="CN1" t="inlineStr">
+      <c r="CS1" t="inlineStr">
         <is>
           <t>informe_bases_existe</t>
         </is>
       </c>
-      <c r="CO1" t="inlineStr">
+      <c r="CT1" t="inlineStr">
         <is>
           <t>informe_bases_numeroid</t>
         </is>
       </c>
-      <c r="CP1" t="inlineStr">
+      <c r="CU1" t="inlineStr">
         <is>
           <t>informe_bases_nombre</t>
         </is>
       </c>
-      <c r="CQ1" t="inlineStr">
+      <c r="CV1" t="inlineStr">
         <is>
           <t>informe_bases_inconveniente</t>
         </is>
       </c>
-      <c r="CR1" t="inlineStr">
+      <c r="CW1" t="inlineStr">
         <is>
           <t>visita_domiciliaria_existe</t>
         </is>
       </c>
-      <c r="CS1" t="inlineStr">
+      <c r="CX1" t="inlineStr">
         <is>
           <t>visita_domiciliaria_numeroid</t>
         </is>
       </c>
-      <c r="CT1" t="inlineStr">
+      <c r="CY1" t="inlineStr">
         <is>
           <t>visita_domiciliaria_nombre</t>
         </is>
       </c>
-      <c r="CU1" t="inlineStr">
+      <c r="CZ1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_existe</t>
         </is>
       </c>
-      <c r="CV1" t="inlineStr">
+      <c r="DA1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_numeroid</t>
         </is>
       </c>
-      <c r="CW1" t="inlineStr">
+      <c r="DB1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_nombre</t>
         </is>
       </c>
-      <c r="CX1" t="inlineStr">
+      <c r="DC1" t="inlineStr">
         <is>
           <t>acuerdo_de_pago_firma</t>
         </is>
       </c>
-      <c r="CY1" t="inlineStr">
+      <c r="DD1" t="inlineStr">
         <is>
           <t>checklist_documentos_existe</t>
         </is>
       </c>
-      <c r="CZ1" t="inlineStr">
+      <c r="DE1" t="inlineStr">
         <is>
           <t>checklist_documentos_numeroid</t>
         </is>
       </c>
-      <c r="DA1" t="inlineStr">
+      <c r="DF1" t="inlineStr">
         <is>
           <t>checklist_documentos_nombre</t>
         </is>
       </c>
-      <c r="DB1" t="inlineStr">
+      <c r="DG1" t="inlineStr">
         <is>
           <t>manual_de_funciones_existe</t>
         </is>
       </c>
-      <c r="DC1" t="inlineStr">
+      <c r="DH1" t="inlineStr">
         <is>
           <t>manual_de_funciones_numeroid</t>
         </is>
       </c>
-      <c r="DD1" t="inlineStr">
+      <c r="DI1" t="inlineStr">
         <is>
           <t>manual_de_funciones_nombre</t>
         </is>
       </c>
-      <c r="DE1" t="inlineStr">
+      <c r="DJ1" t="inlineStr">
         <is>
           <t>compilado_existe</t>
         </is>
       </c>
-      <c r="DF1" t="inlineStr">
+      <c r="DK1" t="inlineStr">
         <is>
           <t>compilado_numeroid</t>
         </is>
       </c>
-      <c r="DG1" t="inlineStr">
+      <c r="DL1" t="inlineStr">
         <is>
           <t>compilado_nombre</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="DM1" t="inlineStr">
         <is>
           <t>otros_existe</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="DN1" t="inlineStr">
         <is>
           <t>otros_numeroid</t>
         </is>
       </c>
-      <c r="DJ1" t="inlineStr">
+      <c r="DO1" t="inlineStr">
         <is>
           <t>otros_nombre</t>
         </is>
       </c>
-      <c r="DK1" t="inlineStr">
+      <c r="DP1" t="inlineStr">
         <is>
           <t>otros_comentario</t>
         </is>
@@ -996,26 +1021,26 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1121877026</v>
+        <v>39576253</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GARCIA LOPEZ NATHALY</t>
+          <t>GUZMAN PAEZ CARMENZA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>/home/real_home/videodrome_estudio/desarrollo/tmp_automatizacion/TEMP/BANCO_DE_BOGOTA_JUNIO_2026/ALEXANDRA BARRERA/1121877026 GARCIA LOPEZ NATHALY</t>
+          <t>/home/real_home/videodrome_estudio/desarrollo/tmp_automatizacion/TEMP/SERGIO_CRUZ/TIGO/39576253 GUZMAN PAEZ CARMENZA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ALEXANDRA BARRERA</t>
+          <t>TIGO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BANCO_DE_BOGOTA_JUNIO_2026</t>
+          <t>SERGIO_CRUZ</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1055,7 +1080,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>20260616</t>
+          <t>20260618</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -1065,72 +1090,48 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>CÓDIGO DE ÉTICA Y CONDUCTA - SAGRILAFT</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>INDUCCIÓN CULTURA SALESLAND</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>PROGRAMA DE TRANSPARENCIA Y ÉTICA EMPRESARIAL</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>ADMINISTRACION DE RECURSOS HUMANOS</t>
+        </is>
+      </c>
       <c r="AE2" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1267,27 +1268,19 @@
       </c>
       <c r="BI2" t="inlineStr">
         <is>
-          <t>445595770</t>
+          <t>0570007271166972</t>
         </is>
       </c>
       <c r="BJ2" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BK2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
       <c r="BM2" t="inlineStr">
         <is>
-          <t>PENSIONES Y CESANTIAS</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="BN2" t="inlineStr">
@@ -1302,19 +1295,11 @@
       </c>
       <c r="BP2" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BQ2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BR2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1322,34 +1307,34 @@
       </c>
       <c r="BT2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
+        <is>
           <t>BACHILLERATO</t>
         </is>
       </c>
-      <c r="BU2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>SIN_DATOS</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="BY2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
       <c r="BZ2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1397,13 +1382,29 @@
       </c>
       <c r="CI2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CJ2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CK2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CL2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="CM2" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="CJ2" t="inlineStr"/>
-      <c r="CK2" t="inlineStr"/>
-      <c r="CL2" t="inlineStr"/>
-      <c r="CM2" t="inlineStr"/>
       <c r="CN2" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1412,46 +1413,30 @@
       <c r="CO2" t="inlineStr"/>
       <c r="CP2" t="inlineStr"/>
       <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr">
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="CS2" t="inlineStr"/>
       <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr">
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr"/>
       <c r="CX2" t="inlineStr"/>
-      <c r="CY2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="CY2" t="inlineStr"/>
       <c r="CZ2" t="inlineStr">
         <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="DA2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="DB2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="DC2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="DA2" t="inlineStr"/>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
       <c r="DD2" t="inlineStr">
         <is>
           <t>SI</t>
@@ -1459,19 +1444,44 @@
       </c>
       <c r="DE2" t="inlineStr">
         <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DF2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DG2" t="inlineStr">
+        <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="DF2" t="inlineStr"/>
-      <c r="DG2" t="inlineStr"/>
-      <c r="DH2" t="inlineStr">
+      <c r="DH2" t="inlineStr"/>
+      <c r="DI2" t="inlineStr"/>
+      <c r="DJ2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DK2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DL2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="DM2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="DI2" t="inlineStr"/>
-      <c r="DJ2" t="inlineStr"/>
-      <c r="DK2" t="inlineStr"/>
+      <c r="DN2" t="inlineStr"/>
+      <c r="DO2" t="inlineStr"/>
+      <c r="DP2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1484,7 +1494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1754,51 +1764,51 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>pension_o_cesantias_tipo</t>
+          <t>estudios_bachillerato</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pension_o_cesantias</t>
+          <t>estudios</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>identificar a qué fondo(s) corresponde la afiliación: PENSIONES, CESANTIAS o PENSIONES Y CESANTIAS</t>
+          <t>verificar si el título obtenido es de bachillerato o secundaria (BACHILLERATO) o de otro nivel superior (OTRO)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>"PENSIONES" o "CESANTIAS" o "PENSIONES Y CESANTIAS"</t>
+          <t>"BACHILLERATO" o "OTRO"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>estudios_bachillerato</t>
+          <t>formatos_para_la_contratacion_hojas</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>estudios</t>
+          <t>formatos_para_la_contratacion</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>verificar si el título obtenido es de bachillerato o secundaria (BACHILLERATO) o de otro nivel superior (OTRO)</t>
+          <t>verificar que el paquete contenga como mínimo 9 hojas en total</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>"BACHILLERATO" o "OTRO"</t>
+          <t>"SI" o "NO"</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>formatos_para_la_contratacion_hojas</t>
+          <t>formatos_para_la_contratacion_firmas</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1808,7 +1818,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>verificar que el paquete contenga como mínimo 9 hojas en total</t>
+          <t>verificar que las 9 hojas estén debidamente diligenciadas y firmadas por el candidato en los espacios correspondientes cuando aplique</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1820,17 +1830,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>formatos_para_la_contratacion_firmas</t>
+          <t>informe_datacredito_moras</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>formatos_para_la_contratacion</t>
+          <t>informe_datacredito</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>verificar que las 9 hojas estén debidamente diligenciadas y firmadas por el candidato en los espacios correspondientes cuando aplique</t>
+          <t>verificar si la persona registra moras o saldos en mora vigentes</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1842,7 +1852,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>informe_datacredito_moras</t>
+          <t>informe_datacredito_demandas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1852,7 +1862,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>verificar si la persona registra moras o saldos en mora vigentes</t>
+          <t>verificar si la persona registra demandas o procesos ejecutivos vigentes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1864,17 +1874,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>informe_datacredito_demandas</t>
+          <t>informe_bases_inconveniente</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>informe_datacredito</t>
+          <t>informe_bases</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>verificar si la persona registra demandas o procesos ejecutivos vigentes</t>
+          <t>verificar si la persona tiene algún inconveniente o reporte negativo que le impida ser contratado</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1886,17 +1896,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>informe_bases_inconveniente</t>
+          <t>acuerdo_de_pago_firma</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>informe_bases</t>
+          <t>acuerdo_de_pago</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>verificar si la persona tiene algún inconveniente o reporte negativo que le impida ser contratado</t>
+          <t>verificar si el acuerdo está firmado explícitamente por quien tiene la deuda</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1908,42 +1918,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>acuerdo_de_pago_firma</t>
+          <t>otros_comentario</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>acuerdo_de_pago</t>
+          <t>otros</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>verificar si el acuerdo está firmado explícitamente por quien tiene la deuda</t>
+          <t>hacer un comentario explicativo sobre qué tipo de documento puede ser</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
-        <is>
-          <t>"SI" o "NO"</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>otros_comentario</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>otros</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>hacer un comentario explicativo sobre qué tipo de documento puede ser</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
         <is>
           <t>string entre comillas "comentario"</t>
         </is>

</xml_diff>